<commit_message>
Fix Furkan Baykusak 29 Sep shift to A
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LsGdck9uUBqMn7Bw6wMhA5
</commit_message>
<xml_diff>
--- a/Personel_Devam_Cizelgesi_Eylul_2026_FURKAN_BAYKUSAK.xlsx
+++ b/Personel_Devam_Cizelgesi_Eylul_2026_FURKAN_BAYKUSAK.xlsx
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C43" s="28" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D43" s="6" t="n"/>
@@ -1824,7 +1824,7 @@
       <c r="H43" s="6" t="n"/>
       <c r="I43" s="28" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="J43" s="9" t="n"/>

</xml_diff>